<commit_message>
Fix normalisation and add validation step
</commit_message>
<xml_diff>
--- a/tests/test_dataset/RepTest_correct.xlsx
+++ b/tests/test_dataset/RepTest_correct.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\llenezet\repositories\Files2DB\tests\test_dataset\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\llenezet\Documents\Repositories\Files2DB\tests\test_dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{308B374E-5D12-41D9-8A6C-63C089CC7EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AB8B1B5-5FCD-42FF-8B99-EF5A7D2A82E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="100">
   <si>
     <t>Eq</t>
   </si>
@@ -80,9 +80,6 @@
     <t>Sep</t>
   </si>
   <si>
-    <t>Del</t>
-  </si>
-  <si>
     <t>DelIn</t>
   </si>
   <si>
@@ -236,9 +233,6 @@
     <t>FilePath</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>Field</t>
   </si>
   <si>
@@ -330,6 +324,15 @@
   </si>
   <si>
     <t>OptColToNotUse</t>
+  </si>
+  <si>
+    <t>Separator</t>
+  </si>
+  <si>
+    <t>DataType</t>
+  </si>
+  <si>
+    <t>DelMatch</t>
   </si>
 </sst>
 </file>
@@ -479,7 +482,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -535,6 +538,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -840,7 +846,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
@@ -865,86 +871,89 @@
     <col min="21" max="21" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" t="s">
         <v>49</v>
       </c>
-      <c r="B1" t="s">
+      <c r="F1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I1" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" t="s">
+        <v>54</v>
+      </c>
+      <c r="K1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" t="s">
+      <c r="L1" t="s">
+        <v>55</v>
+      </c>
+      <c r="M1" t="s">
+        <v>57</v>
+      </c>
+      <c r="N1" t="s">
+        <v>64</v>
+      </c>
+      <c r="O1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G1" t="s">
-        <v>52</v>
-      </c>
-      <c r="H1" t="s">
-        <v>53</v>
-      </c>
-      <c r="I1" t="s">
-        <v>54</v>
-      </c>
-      <c r="J1" t="s">
-        <v>55</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="P1" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q1" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="S1" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="T1" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="U1" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="V1" s="21" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>72</v>
       </c>
-      <c r="L1" t="s">
-        <v>56</v>
-      </c>
-      <c r="M1" t="s">
-        <v>58</v>
-      </c>
-      <c r="N1" t="s">
-        <v>65</v>
-      </c>
-      <c r="O1" t="s">
+      <c r="B2" t="s">
         <v>73</v>
       </c>
-      <c r="P1" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q1" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="S1" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="T1" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="U1" s="14" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>74</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>75</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>76</v>
-      </c>
-      <c r="D2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E2" t="s">
-        <v>78</v>
       </c>
       <c r="F2">
         <v>4</v>
@@ -956,16 +965,16 @@
         <v>3</v>
       </c>
       <c r="I2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J2" t="s">
         <v>62</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
+        <v>77</v>
+      </c>
+      <c r="L2" t="s">
         <v>63</v>
-      </c>
-      <c r="K2" t="s">
-        <v>79</v>
-      </c>
-      <c r="L2" t="s">
-        <v>64</v>
       </c>
       <c r="P2" s="10">
         <v>1</v>
@@ -977,15 +986,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" t="s">
         <v>80</v>
-      </c>
-      <c r="C3" t="s">
-        <v>81</v>
-      </c>
-      <c r="D3" t="s">
-        <v>82</v>
       </c>
       <c r="F3">
         <v>2</v>
@@ -997,16 +1006,16 @@
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1036,75 +1045,75 @@
   <sheetData>
     <row r="1" spans="1:15" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="H1" s="18" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="I1" s="18" t="s">
-        <v>67</v>
+        <v>98</v>
       </c>
       <c r="J1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="L1" s="7" t="s">
-        <v>32</v>
-      </c>
       <c r="M1" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="N1" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="N1" s="18" t="s">
-        <v>88</v>
-      </c>
       <c r="O1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="C2" s="16" t="s">
         <v>34</v>
-      </c>
-      <c r="C2" s="16" t="s">
-        <v>35</v>
       </c>
       <c r="D2" s="17"/>
       <c r="E2" s="17"/>
       <c r="F2" s="17"/>
       <c r="G2" s="16" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I2" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" s="17" t="s">
         <v>36</v>
-      </c>
-      <c r="J2" s="17" t="s">
-        <v>37</v>
       </c>
       <c r="L2" s="9"/>
       <c r="M2" s="16"/>
@@ -1115,7 +1124,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C3" s="16"/>
       <c r="D3" s="17"/>
@@ -1124,10 +1133,10 @@
       <c r="G3" s="16"/>
       <c r="H3" s="20"/>
       <c r="I3" s="19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J3" s="17" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L3" s="9"/>
       <c r="M3" s="16"/>
@@ -1138,21 +1147,21 @@
         <v>8</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C4" s="16"/>
       <c r="D4" s="17"/>
       <c r="E4" s="17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F4" s="17"/>
       <c r="G4" s="16"/>
       <c r="H4" s="20"/>
       <c r="I4" s="19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J4" s="17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L4" s="9"/>
       <c r="M4" s="16"/>
@@ -1160,26 +1169,26 @@
     </row>
     <row r="5" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="16" t="s">
         <v>42</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>43</v>
       </c>
       <c r="D5" s="17"/>
       <c r="E5" s="17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F5" s="17"/>
       <c r="G5" s="16"/>
       <c r="H5" s="20"/>
       <c r="I5" s="19" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J5" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K5" s="10">
         <v>111111</v>
@@ -1192,77 +1201,77 @@
     </row>
     <row r="6" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D6" s="17"/>
       <c r="E6" s="17"/>
       <c r="F6" s="17"/>
       <c r="G6" s="16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H6" s="20"/>
       <c r="I6" s="19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L6" s="9"/>
       <c r="N6" s="20"/>
     </row>
     <row r="7" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" s="16"/>
       <c r="D7" s="17"/>
       <c r="E7" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F7" s="17"/>
       <c r="G7" s="16"/>
       <c r="H7" s="20"/>
       <c r="I7" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J7" s="17"/>
       <c r="L7" s="9"/>
       <c r="M7" s="17" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="N7" s="20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C8" s="16"/>
       <c r="D8" s="17"/>
       <c r="E8" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F8" s="17"/>
       <c r="G8" s="16"/>
       <c r="H8" s="20"/>
       <c r="I8" s="19" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J8" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K8" s="10">
         <v>111111111111111</v>
@@ -1275,24 +1284,24 @@
     </row>
     <row r="9" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="17"/>
       <c r="E9" s="17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F9" s="17"/>
       <c r="G9" s="16"/>
       <c r="H9" s="20"/>
       <c r="I9" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J9" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="K9" s="10">
         <v>6</v>
@@ -1305,10 +1314,10 @@
     </row>
     <row r="10" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="17"/>
@@ -1317,23 +1326,23 @@
       <c r="G10" s="16"/>
       <c r="H10" s="20"/>
       <c r="I10" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J10" s="17"/>
       <c r="L10" s="9"/>
       <c r="M10" s="16" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="N10" s="19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="17"/>
@@ -1342,10 +1351,10 @@
       <c r="G11" s="16"/>
       <c r="H11" s="20"/>
       <c r="I11" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J11" s="17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L11" s="9"/>
       <c r="N11" s="19"/>
@@ -1380,7 +1389,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1450,7 +1459,7 @@
         <v>13</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>